<commit_message>
MA dependances FrCore + MAJ RC documentReference (#115) e1905721f09631a9a6b6053e42449dd125998abb
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-documentreference.xlsx
+++ b/main/ig/StructureDefinition-tddui-documentreference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2537" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2537" uniqueCount="533">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-19T07:50:19+00:00</t>
+    <t>2024-06-20T09:03:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -868,7 +868,7 @@
     <t>DocumentReference.subject</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Patient)
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient)
 </t>
   </si>
   <si>
@@ -1659,10 +1659,6 @@
   </si>
   <si>
     <t>DocumentReference.context.sourcePatientInfo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference(http://interopsante.org/fhir/StructureDefinition/FrPatient)
-</t>
   </si>
   <si>
     <t>Référence vers la ressource Patient titulaire du dossier.</t>
@@ -9725,13 +9721,13 @@
         <v>80</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="L63" t="s" s="2">
         <v>521</v>
       </c>
-      <c r="L63" t="s" s="2">
+      <c r="M63" t="s" s="2">
         <v>522</v>
-      </c>
-      <c r="M63" t="s" s="2">
-        <v>523</v>
       </c>
       <c r="N63" t="s" s="2">
         <v>274</v>
@@ -9817,15 +9813,15 @@
         <v>80</v>
       </c>
       <c r="AQ63" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9848,16 +9844,16 @@
         <v>80</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>525</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>527</v>
       </c>
-      <c r="M64" t="s" s="2">
+      <c r="N64" t="s" s="2">
         <v>528</v>
-      </c>
-      <c r="N64" t="s" s="2">
-        <v>529</v>
       </c>
       <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
@@ -9907,7 +9903,7 @@
         <v>80</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>81</v>
@@ -9925,22 +9921,22 @@
         <v>80</v>
       </c>
       <c r="AL64" t="s" s="2">
+        <v>529</v>
+      </c>
+      <c r="AM64" t="s" s="2">
         <v>530</v>
       </c>
-      <c r="AM64" t="s" s="2">
+      <c r="AN64" t="s" s="2">
         <v>531</v>
       </c>
-      <c r="AN64" t="s" s="2">
+      <c r="AO64" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP64" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ64" t="s" s="2">
         <v>532</v>
-      </c>
-      <c r="AO64" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP64" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ64" t="s" s="2">
-        <v>533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>